<commit_message>
[dados 28/08] Planilha Mestra atualizada: Registro_Vendas com 3 vendas novas (L2460-CP 19/08, Q3060-A 3un 20/08, PXM 26/08) — 42 linhas de dados, TOTAIS recalculado
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Micro\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Micro\Desktop\amazon\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1747" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="530">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1636,7 +1636,7 @@
     <numFmt numFmtId="165" formatCode="&quot;R$ &quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1649,45 +1649,45 @@
       <sz val="13"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1696,6 +1696,19 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1769,7 +1782,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1831,6 +1844,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13649,7 +13664,7 @@
         <v>814.08</v>
       </c>
       <c r="I199" s="12">
-        <f t="shared" ref="I199:I262" si="19">IF(OR(G199="",H199=""),"",G199/H199)</f>
+        <f t="shared" ref="I199:I232" si="19">IF(OR(G199="",H199=""),"",G199/H199)</f>
         <v>0.13562549135220126</v>
       </c>
       <c r="J199" s="13">
@@ -13661,19 +13676,19 @@
         <v>233</v>
       </c>
       <c r="L199" s="13">
-        <f t="shared" ref="L199:L262" si="20">IF(OR(J199="",K199=""),"",J199-K199)</f>
+        <f t="shared" ref="L199:L232" si="20">IF(OR(J199="",K199=""),"",J199-K199)</f>
         <v>0</v>
       </c>
       <c r="M199" s="13">
-        <f t="shared" ref="M199:M262" si="21">IF(OR(H199="",F199="",G199=""),"",H199-G199-F199-H199*$B$3+IF(L199="",0,L199))</f>
+        <f t="shared" ref="M199:M232" si="21">IF(OR(H199="",F199="",G199=""),"",H199-G199-F199-H199*$B$3+IF(L199="",0,L199))</f>
         <v>222.09200000000004</v>
       </c>
       <c r="N199" s="12">
-        <f t="shared" ref="N199:N262" si="22">IF(OR(M199="",H199=0,H199=""),"",M199/H199)</f>
+        <f t="shared" ref="N199:N232" si="22">IF(OR(M199="",H199=0,H199=""),"",M199/H199)</f>
         <v>0.27281348270440253</v>
       </c>
       <c r="O199" s="22" t="str">
-        <f t="shared" ref="O199:O262" si="23">IF(N199="","",IF(N199&lt;0,"PREJUÍZO",IF(N199&lt;0.1,"CRÍTICO (&lt;10%)",IF(N199&lt;0.15,"ABAIXO DA META (10-15%)",IF(N199&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
+        <f t="shared" ref="O199:O232" si="23">IF(N199="","",IF(N199&lt;0,"PREJUÍZO",IF(N199&lt;0.1,"CRÍTICO (&lt;10%)",IF(N199&lt;0.15,"ABAIXO DA META (10-15%)",IF(N199&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="P199" s="23"/>
@@ -18128,151 +18143,183 @@
       <c r="R44" s="19"/>
     </row>
     <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="32"/>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="20" t="str">
+      <c r="A45" s="32">
+        <v>46253</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="C45" s="19">
+        <v>1</v>
+      </c>
+      <c r="D45" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="E45" s="20">
         <f>IF($B45="","",INDEX(Simulador!$D$7:$D$232,MATCH($B45,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>335.68</v>
       </c>
       <c r="F45" s="20"/>
-      <c r="G45" s="13" t="str">
+      <c r="G45" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>335.68</v>
       </c>
       <c r="H45" s="8" t="str">
         <f>IF($B45="","",INDEX(Simulador!$B$7:$B$232,MATCH($B45,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I45" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I45" s="13">
         <f>IF(OR(H45="",$D45=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D45,Ref_Frete!$A$2:$A$54,0),IF(H45="Pequenos",2,IF(H45="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20" t="str">
+        <v>158</v>
+      </c>
+      <c r="J45" s="20">
+        <v>61.25</v>
+      </c>
+      <c r="K45" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L45" s="13" t="str">
+        <v>66.650000000000006</v>
+      </c>
+      <c r="L45" s="13">
         <f>IF(OR($B45="",$C45=""),"",$C45*INDEX(Simulador!$F$7:$F$232,MATCH($B45,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M45" s="13" t="str">
+        <v>172.67</v>
+      </c>
+      <c r="M45" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N45" s="35" t="str">
+        <v>33.568000000000005</v>
+      </c>
+      <c r="N45" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O45" s="12" t="str">
+        <v>159.54199999999997</v>
+      </c>
+      <c r="O45" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.47528002859866531</v>
       </c>
       <c r="P45" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q45" s="19"/>
       <c r="R45" s="19"/>
     </row>
     <row r="46" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="32"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="20" t="str">
+      <c r="A46" s="32">
+        <v>46254</v>
+      </c>
+      <c r="B46" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" s="19">
+        <v>3</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E46" s="20">
         <f>IF($B46="","",INDEX(Simulador!$D$7:$D$232,MATCH($B46,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F46" s="20"/>
-      <c r="G46" s="13" t="str">
+        <v>580.52</v>
+      </c>
+      <c r="F46" s="20">
+        <v>87.08</v>
+      </c>
+      <c r="G46" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1654.48</v>
       </c>
       <c r="H46" s="8" t="str">
         <f>IF($B46="","",INDEX(Simulador!$B$7:$B$232,MATCH($B46,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I46" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I46" s="13">
         <f>IF(OR(H46="",$D46=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D46,Ref_Frete!$A$2:$A$54,0),IF(H46="Pequenos",2,IF(H46="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20" t="str">
+        <v>34.9</v>
+      </c>
+      <c r="J46" s="20">
+        <v>0</v>
+      </c>
+      <c r="K46" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L46" s="13" t="str">
+        <v>228.07</v>
+      </c>
+      <c r="L46" s="13">
         <f>IF(OR($B46="",$C46=""),"",$C46*INDEX(Simulador!$F$7:$F$232,MATCH($B46,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M46" s="13" t="str">
+        <v>833.25</v>
+      </c>
+      <c r="M46" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N46" s="35" t="str">
+        <v>165.44800000000001</v>
+      </c>
+      <c r="N46" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O46" s="12" t="str">
+        <v>462.61200000000019</v>
+      </c>
+      <c r="O46" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.27961172090324465</v>
       </c>
       <c r="P46" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q46" s="19"/>
       <c r="R46" s="19"/>
     </row>
     <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="32"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="20" t="str">
+      <c r="A47" s="32">
+        <v>46260</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" s="19">
+        <v>1</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>384</v>
+      </c>
+      <c r="E47" s="20">
         <f>IF($B47="","",INDEX(Simulador!$D$7:$D$232,MATCH($B47,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>203.54</v>
       </c>
       <c r="F47" s="20"/>
-      <c r="G47" s="13" t="str">
+      <c r="G47" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>203.54</v>
       </c>
       <c r="H47" s="8" t="str">
         <f>IF($B47="","",INDEX(Simulador!$B$7:$B$232,MATCH($B47,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I47" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I47" s="13">
         <f>IF(OR(H47="",$D47=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D47,Ref_Frete!$A$2:$A$54,0),IF(H47="Pequenos",2,IF(H47="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J47" s="20"/>
-      <c r="K47" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J47" s="20">
+        <v>18.079999999999998</v>
+      </c>
+      <c r="K47" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L47" s="13" t="str">
+        <v>30.84</v>
+      </c>
+      <c r="L47" s="13">
         <f>IF(OR($B47="",$C47=""),"",$C47*INDEX(Simulador!$F$7:$F$232,MATCH($B47,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M47" s="13" t="str">
+        <v>102.8</v>
+      </c>
+      <c r="M47" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N47" s="35" t="str">
+        <v>20.353999999999999</v>
+      </c>
+      <c r="N47" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O47" s="12" t="str">
+        <v>56.366000000000014</v>
+      </c>
+      <c r="O47" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.27692836788837583</v>
       </c>
       <c r="P47" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q47" s="19"/>
       <c r="R47" s="19"/>
@@ -18295,7 +18342,7 @@
         <f>IF($B48="","",INDEX(Simulador!$B$7:$B$232,MATCH($B48,Simulador!$A$7:$A$232,0)))</f>
         <v/>
       </c>
-      <c r="I48" s="13" t="str">
+      <c r="I48" s="47" t="str">
         <f>IF(OR(H48="",$D48=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D48,Ref_Frete!$A$2:$A$54,0),IF(H48="Pequenos",2,IF(H48="Medios",4,6))))</f>
         <v/>
       </c>
@@ -18350,7 +18397,7 @@
         <v/>
       </c>
       <c r="J49" s="20"/>
-      <c r="K49" s="20" t="str">
+      <c r="K49" s="48" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
@@ -18387,7 +18434,7 @@
         <v/>
       </c>
       <c r="F50" s="20"/>
-      <c r="G50" s="13" t="str">
+      <c r="G50" s="47" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -20988,7 +21035,7 @@
       </c>
       <c r="F102" s="20"/>
       <c r="G102" s="13" t="str">
-        <f t="shared" ref="G102:G133" si="18">IF(OR($B102="",$C102=""),"",$C102*E102-IF(F102="",0,F102))</f>
+        <f t="shared" ref="G102:G107" si="18">IF(OR($B102="",$C102=""),"",$C102*E102-IF(F102="",0,F102))</f>
         <v/>
       </c>
       <c r="H102" s="8" t="str">
@@ -21013,15 +21060,15 @@
         <v/>
       </c>
       <c r="N102" s="35" t="str">
-        <f t="shared" ref="N102:N133" si="20">IF(OR(G102="",J102=""),"",G102+IF(I102="",0,I102)-J102-K102-L102-M102)</f>
+        <f t="shared" ref="N102:N107" si="20">IF(OR(G102="",J102=""),"",G102+IF(I102="",0,I102)-J102-K102-L102-M102)</f>
         <v/>
       </c>
       <c r="O102" s="12" t="str">
-        <f t="shared" ref="O102:O133" si="21">IF(OR(N102="",G102=0,G102=""),"",N102/G102)</f>
+        <f t="shared" ref="O102:O107" si="21">IF(OR(N102="",G102=0,G102=""),"",N102/G102)</f>
         <v/>
       </c>
       <c r="P102" s="22" t="str">
-        <f t="shared" ref="P102:P133" si="22">IF(O102="","",IF(O102&lt;0,"PREJUÍZO",IF(O102&lt;0.1,"CRÍTICO (&lt;10%)",IF(O102&lt;0.15,"ABAIXO DA META (10-15%)",IF(O102&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
+        <f t="shared" ref="P102:P107" si="22">IF(O102="","",IF(O102&lt;0,"PREJUÍZO",IF(O102&lt;0.1,"CRÍTICO (&lt;10%)",IF(O102&lt;0.15,"ABAIXO DA META (10-15%)",IF(O102&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
         <v/>
       </c>
       <c r="Q102" s="19"/>
@@ -21283,27 +21330,27 @@
       </c>
       <c r="G108" s="38">
         <f>SUM(G6:G107)</f>
-        <v>17983.300000000007</v>
+        <v>20177.000000000007</v>
       </c>
       <c r="K108" s="38">
         <f>SUM(K6:K107)</f>
-        <v>2730.18</v>
+        <v>3055.7400000000002</v>
       </c>
       <c r="L108" s="38">
         <f>SUM(L6:L107)</f>
-        <v>9527.8200000000015</v>
+        <v>10636.54</v>
       </c>
       <c r="M108" s="38">
         <f>SUM(M6:M107)</f>
-        <v>1798.3300000000006</v>
+        <v>2017.7000000000007</v>
       </c>
       <c r="N108" s="38">
         <f>SUM(N6:N107)</f>
-        <v>4365.1100000000006</v>
+        <v>5043.630000000001</v>
       </c>
       <c r="O108" s="39">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.2427313118281961</v>
+        <v>0.24996927194330174</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -21317,7 +21364,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">

</xml_diff>

<commit_message>
[dados 31/08] Planilha Mestra atualizada: vendas PXP 29/08 e L2025-T 30/08 no Registro_Vendas — 44 linhas de dados, TOTAIS R$ 20.477,79 / margem 25,1%
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1753" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="530">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -18325,101 +18325,121 @@
       <c r="R47" s="19"/>
     </row>
     <row r="48" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="32"/>
-      <c r="B48" s="19"/>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="20" t="str">
+      <c r="A48" s="32">
+        <v>46263</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C48" s="19">
+        <v>1</v>
+      </c>
+      <c r="D48" s="19" t="s">
+        <v>384</v>
+      </c>
+      <c r="E48" s="20">
         <f>IF($B48="","",INDEX(Simulador!$D$7:$D$232,MATCH($B48,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>167.89</v>
       </c>
       <c r="F48" s="20"/>
-      <c r="G48" s="13" t="str">
+      <c r="G48" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>167.89</v>
       </c>
       <c r="H48" s="8" t="str">
         <f>IF($B48="","",INDEX(Simulador!$B$7:$B$232,MATCH($B48,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I48" s="47" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I48" s="47">
         <f>IF(OR(H48="",$D48=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D48,Ref_Frete!$A$2:$A$54,0),IF(H48="Pequenos",2,IF(H48="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J48" s="20"/>
-      <c r="K48" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J48" s="20">
+        <v>14.69</v>
+      </c>
+      <c r="K48" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L48" s="13" t="str">
+        <v>26.03</v>
+      </c>
+      <c r="L48" s="13">
         <f>IF(OR($B48="",$C48=""),"",$C48*INDEX(Simulador!$F$7:$F$232,MATCH($B48,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M48" s="13" t="str">
+        <v>84.79</v>
+      </c>
+      <c r="M48" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N48" s="35" t="str">
+        <v>16.788999999999998</v>
+      </c>
+      <c r="N48" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O48" s="12" t="str">
+        <v>50.490999999999985</v>
+      </c>
+      <c r="O48" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.30073857883137761</v>
       </c>
       <c r="P48" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q48" s="19"/>
       <c r="R48" s="19"/>
     </row>
     <row r="49" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="32"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="20" t="str">
+      <c r="A49" s="32">
+        <v>46264</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C49" s="19">
+        <v>1</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E49" s="20">
         <f>IF($B49="","",INDEX(Simulador!$D$7:$D$232,MATCH($B49,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F49" s="20"/>
-      <c r="G49" s="13" t="str">
+      <c r="G49" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="H49" s="8" t="str">
         <f>IF($B49="","",INDEX(Simulador!$B$7:$B$232,MATCH($B49,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I49" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I49" s="13">
         <f>IF(OR(H49="",$D49=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D49,Ref_Frete!$A$2:$A$54,0),IF(H49="Pequenos",2,IF(H49="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J49" s="20"/>
-      <c r="K49" s="48" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J49" s="20">
+        <v>15.65</v>
+      </c>
+      <c r="K49" s="48">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L49" s="13" t="str">
+        <v>21.3</v>
+      </c>
+      <c r="L49" s="13">
         <f>IF(OR($B49="",$C49=""),"",$C49*INDEX(Simulador!$F$7:$F$232,MATCH($B49,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M49" s="13" t="str">
+        <v>63.11</v>
+      </c>
+      <c r="M49" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N49" s="35" t="str">
+        <v>13.290000000000001</v>
+      </c>
+      <c r="N49" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O49" s="12" t="str">
+        <v>44.45000000000001</v>
+      </c>
+      <c r="O49" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.33446200150489097</v>
       </c>
       <c r="P49" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q49" s="19"/>
       <c r="R49" s="19"/>
@@ -21330,27 +21350,27 @@
       </c>
       <c r="G108" s="38">
         <f>SUM(G6:G107)</f>
-        <v>20177.000000000007</v>
+        <v>20477.790000000008</v>
       </c>
       <c r="K108" s="38">
         <f>SUM(K6:K107)</f>
-        <v>3055.7400000000002</v>
+        <v>3103.0700000000006</v>
       </c>
       <c r="L108" s="38">
         <f>SUM(L6:L107)</f>
-        <v>10636.54</v>
+        <v>10784.440000000002</v>
       </c>
       <c r="M108" s="38">
         <f>SUM(M6:M107)</f>
-        <v>2017.7000000000007</v>
+        <v>2047.7790000000007</v>
       </c>
       <c r="N108" s="38">
         <f>SUM(N6:N107)</f>
-        <v>5043.630000000001</v>
+        <v>5138.5710000000008</v>
       </c>
       <c r="O108" s="39">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.24996927194330174</v>
+        <v>0.25093386542200102</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[dados 01/09] Mestra: 4 vendas novas lancadas (L2025-T 2un MS, L2450-AML 3un PE, L2025-T 1un MG em 31/08; L2030-T 1un GO em 01/09) — 48 linhas, receita R$ 21.799,32
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_2.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1765" uniqueCount="530">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -18445,201 +18445,241 @@
       <c r="R49" s="19"/>
     </row>
     <row r="50" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="32"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="20" t="str">
+      <c r="A50" s="32">
+        <v>46265</v>
+      </c>
+      <c r="B50" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" s="19">
+        <v>2</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="E50" s="20">
         <f>IF($B50="","",INDEX(Simulador!$D$7:$D$232,MATCH($B50,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F50" s="20"/>
-      <c r="G50" s="47" t="str">
+      <c r="G50" s="47">
         <f t="shared" si="6"/>
-        <v/>
+        <v>265.8</v>
       </c>
       <c r="H50" s="8" t="str">
         <f>IF($B50="","",INDEX(Simulador!$B$7:$B$232,MATCH($B50,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I50" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I50" s="13">
         <f>IF(OR(H50="",$D50=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D50,Ref_Frete!$A$2:$A$54,0),IF(H50="Pequenos",2,IF(H50="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20" t="str">
+        <v>43</v>
+      </c>
+      <c r="J50" s="20">
+        <v>20.98</v>
+      </c>
+      <c r="K50" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L50" s="13" t="str">
+        <v>41.69</v>
+      </c>
+      <c r="L50" s="13">
         <f>IF(OR($B50="",$C50=""),"",$C50*INDEX(Simulador!$F$7:$F$232,MATCH($B50,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M50" s="13" t="str">
+        <v>126.22</v>
+      </c>
+      <c r="M50" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N50" s="35" t="str">
+        <v>26.580000000000002</v>
+      </c>
+      <c r="N50" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O50" s="12" t="str">
+        <v>93.33</v>
+      </c>
+      <c r="O50" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.35112866817155752</v>
       </c>
       <c r="P50" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q50" s="19"/>
       <c r="R50" s="19"/>
     </row>
     <row r="51" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="32"/>
-      <c r="B51" s="19"/>
-      <c r="C51" s="19"/>
-      <c r="D51" s="19"/>
-      <c r="E51" s="20" t="str">
+      <c r="A51" s="32">
+        <v>46265</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C51" s="19">
+        <v>3</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="E51" s="20">
         <f>IF($B51="","",INDEX(Simulador!$D$7:$D$232,MATCH($B51,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>259.89999999999998</v>
       </c>
       <c r="F51" s="20"/>
-      <c r="G51" s="13" t="str">
+      <c r="G51" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>779.69999999999993</v>
       </c>
       <c r="H51" s="8" t="str">
         <f>IF($B51="","",INDEX(Simulador!$B$7:$B$232,MATCH($B51,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I51" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I51" s="13">
         <f>IF(OR(H51="",$D51=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D51,Ref_Frete!$A$2:$A$54,0),IF(H51="Pequenos",2,IF(H51="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20" t="str">
+        <v>70</v>
+      </c>
+      <c r="J51" s="20">
+        <v>102.9</v>
+      </c>
+      <c r="K51" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L51" s="13" t="str">
+        <v>114.71</v>
+      </c>
+      <c r="L51" s="13">
         <f>IF(OR($B51="",$C51=""),"",$C51*INDEX(Simulador!$F$7:$F$232,MATCH($B51,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M51" s="13" t="str">
+        <v>418.47</v>
+      </c>
+      <c r="M51" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N51" s="35" t="str">
+        <v>77.97</v>
+      </c>
+      <c r="N51" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O51" s="12" t="str">
+        <v>135.64999999999989</v>
+      </c>
+      <c r="O51" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.17397717070668192</v>
       </c>
       <c r="P51" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>DENTRO DA META (15-20%)</v>
       </c>
       <c r="Q51" s="19"/>
       <c r="R51" s="19"/>
     </row>
     <row r="52" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="32"/>
-      <c r="B52" s="19"/>
-      <c r="C52" s="19"/>
-      <c r="D52" s="19"/>
-      <c r="E52" s="20" t="str">
+      <c r="A52" s="32">
+        <v>46265</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" s="19">
+        <v>1</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>384</v>
+      </c>
+      <c r="E52" s="20">
         <f>IF($B52="","",INDEX(Simulador!$D$7:$D$232,MATCH($B52,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F52" s="20"/>
-      <c r="G52" s="13" t="str">
+      <c r="G52" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="H52" s="8" t="str">
         <f>IF($B52="","",INDEX(Simulador!$B$7:$B$232,MATCH($B52,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I52" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I52" s="13">
         <f>IF(OR(H52="",$D52=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D52,Ref_Frete!$A$2:$A$54,0),IF(H52="Pequenos",2,IF(H52="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J52" s="20">
+        <v>14.3</v>
+      </c>
+      <c r="K52" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L52" s="13" t="str">
+        <v>21.3</v>
+      </c>
+      <c r="L52" s="13">
         <f>IF(OR($B52="",$C52=""),"",$C52*INDEX(Simulador!$F$7:$F$232,MATCH($B52,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M52" s="13" t="str">
+        <v>63.11</v>
+      </c>
+      <c r="M52" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N52" s="35" t="str">
+        <v>13.290000000000001</v>
+      </c>
+      <c r="N52" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O52" s="12" t="str">
+        <v>45.800000000000004</v>
+      </c>
+      <c r="O52" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.34462001504890899</v>
       </c>
       <c r="P52" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q52" s="19"/>
       <c r="R52" s="19"/>
     </row>
     <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="32"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="20" t="str">
+      <c r="A53" s="32">
+        <v>46266</v>
+      </c>
+      <c r="B53" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" s="19">
+        <v>1</v>
+      </c>
+      <c r="D53" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="E53" s="20">
         <f>IF($B53="","",INDEX(Simulador!$D$7:$D$232,MATCH($B53,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>143.13</v>
       </c>
       <c r="F53" s="20"/>
-      <c r="G53" s="13" t="str">
+      <c r="G53" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>143.13</v>
       </c>
       <c r="H53" s="8" t="str">
         <f>IF($B53="","",INDEX(Simulador!$B$7:$B$232,MATCH($B53,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I53" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I53" s="13">
         <f>IF(OR(H53="",$D53=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D53,Ref_Frete!$A$2:$A$54,0),IF(H53="Pequenos",2,IF(H53="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20" t="str">
+        <v>42</v>
+      </c>
+      <c r="J53" s="20">
+        <v>19.45</v>
+      </c>
+      <c r="K53" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L53" s="13" t="str">
+        <v>24.99</v>
+      </c>
+      <c r="L53" s="13">
         <f>IF(OR($B53="",$C53=""),"",$C53*INDEX(Simulador!$F$7:$F$232,MATCH($B53,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M53" s="13" t="str">
+        <v>69.27</v>
+      </c>
+      <c r="M53" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N53" s="35" t="str">
+        <v>14.313000000000001</v>
+      </c>
+      <c r="N53" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O53" s="12" t="str">
+        <v>57.106999999999999</v>
+      </c>
+      <c r="O53" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.39898693495423743</v>
       </c>
       <c r="P53" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q53" s="19"/>
       <c r="R53" s="19"/>
@@ -21350,27 +21390,27 @@
       </c>
       <c r="G108" s="38">
         <f>SUM(G6:G107)</f>
-        <v>20477.790000000008</v>
+        <v>21799.320000000011</v>
       </c>
       <c r="K108" s="38">
         <f>SUM(K6:K107)</f>
-        <v>3103.0700000000006</v>
+        <v>3305.7600000000007</v>
       </c>
       <c r="L108" s="38">
         <f>SUM(L6:L107)</f>
-        <v>10784.440000000002</v>
+        <v>11461.510000000002</v>
       </c>
       <c r="M108" s="38">
         <f>SUM(M6:M107)</f>
-        <v>2047.7790000000007</v>
+        <v>2179.9320000000007</v>
       </c>
       <c r="N108" s="38">
         <f>SUM(N6:N107)</f>
-        <v>5138.5710000000008</v>
+        <v>5470.4580000000005</v>
       </c>
       <c r="O108" s="39">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25093386542200102</v>
+        <v>0.25094626804872805</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>